<commit_message>
fix(clues): separar Hospital General viejo (QTSSA001752) del Nuevo Hospital General NHGQ (QTSSA002901)
La plantilla SINBA (hoja DATOS), el catalogo de unidades y los scripts de
requisiciones tenian QTSSA002901 en el Hospital General de Queretaro viejo. Ahora
QTSSA001752 = HGQ viejo (inactivo) y QTSSA002901 = NHGQ (activo, municipio NHG).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SINBA-VER_26_2026.xlsx
+++ b/SINBA-VER_26_2026.xlsx
@@ -72,7 +72,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1531" uniqueCount="967">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1531" uniqueCount="968">
   <si>
     <t>Total</t>
   </si>
@@ -3971,6 +3971,9 @@
   </si>
   <si>
     <t>QTSSA013034</t>
+  </si>
+  <si>
+    <t>QTSSA001752</t>
   </si>
 </sst>
 </file>
@@ -12146,7 +12149,7 @@
         <v>424</v>
       </c>
       <c r="D4" s="82" t="s">
-        <v>275</v>
+        <v>967</v>
       </c>
       <c r="E4" s="84"/>
       <c r="F4" t="s">
@@ -12326,7 +12329,7 @@
         <v>424</v>
       </c>
       <c r="H13" t="s">
-        <v>275</v>
+        <v>967</v>
       </c>
       <c r="I13" t="s">
         <v>239</v>

</xml_diff>